<commit_message>
added: extra options for DataStores: --rows ROWS and --filestore
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F14FBA2-BD66-46F6-8AE2-A52C7C15C5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48AF1768-1ADE-4CC0-8EDE-EE8FA89794F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1755" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="271">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -950,6 +950,9 @@
   </si>
   <si>
     <t>Field accepting GeoJSON (WKB hexadecimal preferred), in WGS84 coordinate system (4326). To convert from an existing EPSG, use argument --epsg-src in the Options column of the field</t>
+  </si>
+  <si>
+    <t>--rows 45</t>
   </si>
 </sst>
 </file>
@@ -1031,7 +1034,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1097,6 +1100,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -2594,6 +2598,9 @@
       <c r="H3" t="s">
         <v>15</v>
       </c>
+      <c r="L3" s="23" t="s">
+        <v>270</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">

</xml_diff>

<commit_message>
fixed: compatibility with CKAN 2.11.5
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48AF1768-1ADE-4CC0-8EDE-EE8FA89794F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{464EE3CE-8388-464C-B9A2-DE1DD6F8A970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
   <sheets>
     <sheet name="ckan" sheetId="7" r:id="rId1"/>
@@ -294,9 +294,6 @@
     <t>builder-example-py</t>
   </si>
   <si>
-    <t>Example package to build with package builder from Python ckan_requests.builder</t>
-  </si>
-  <si>
     <t>0.0.0</t>
   </si>
   <si>
@@ -953,6 +950,9 @@
   </si>
   <si>
     <t>--rows 45</t>
+  </si>
+  <si>
+    <t>Example package to build with package builder from Python ckanapi_harvesters.builder</t>
   </si>
 </sst>
 </file>
@@ -1034,7 +1034,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1076,6 +1076,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1100,7 +1101,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1457,88 +1458,88 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C7" t="s">
         <v>178</v>
-      </c>
-      <c r="C7" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B10">
         <v>1000</v>
       </c>
       <c r="C10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B11">
         <v>0.1</v>
       </c>
       <c r="C11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -1559,40 +1560,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+    </row>
+    <row r="2" spans="1:3" ht="102" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-    </row>
-    <row r="2" spans="1:3" ht="102" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
     </row>
     <row r="3" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
+      <c r="A3" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>102</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>103</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>3</v>
@@ -1600,86 +1601,86 @@
     </row>
     <row r="7" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="C7" s="19"/>
+      <c r="C7" s="20"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>200</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="20"/>
+      <c r="B13" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13" s="21"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>53</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1690,7 +1691,7 @@
         <v>9</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1701,7 +1702,7 @@
         <v>3</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1712,7 +1713,7 @@
         <v>11</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="60" x14ac:dyDescent="0.25">
@@ -1723,7 +1724,7 @@
         <v>24</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="75" x14ac:dyDescent="0.25">
@@ -1734,7 +1735,7 @@
         <v>46</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -1745,7 +1746,7 @@
         <v>10</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1756,7 +1757,7 @@
         <v>23</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1767,7 +1768,7 @@
         <v>32</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -1778,7 +1779,7 @@
         <v>51</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1789,7 +1790,7 @@
         <v>26</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1800,7 +1801,7 @@
         <v>27</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1811,7 +1812,7 @@
         <v>28</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1822,7 +1823,7 @@
         <v>29</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -1830,139 +1831,139 @@
         <v>53</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="B29" s="19" t="s">
-        <v>143</v>
-      </c>
-      <c r="C29" s="19"/>
+        <v>108</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>142</v>
+      </c>
+      <c r="C29" s="20"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="195" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="195" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B35" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>178</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B38" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="C38" s="9" t="s">
         <v>259</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="C40" s="20"/>
+      <c r="B40" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="C40" s="21"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
@@ -1972,7 +1973,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -1983,7 +1984,7 @@
         <v>3</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -1994,7 +1995,7 @@
         <v>2</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -2005,7 +2006,7 @@
         <v>46</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="375" x14ac:dyDescent="0.25">
@@ -2016,7 +2017,7 @@
         <v>30</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -2024,10 +2025,10 @@
         <v>54</v>
       </c>
       <c r="B46" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="75" x14ac:dyDescent="0.25">
@@ -2038,7 +2039,7 @@
         <v>4</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="90" x14ac:dyDescent="0.25">
@@ -2049,7 +2050,7 @@
         <v>47</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -2060,7 +2061,7 @@
         <v>48</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="60" x14ac:dyDescent="0.25">
@@ -2068,10 +2069,10 @@
         <v>54</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -2079,10 +2080,10 @@
         <v>54</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -2090,114 +2091,114 @@
         <v>54</v>
       </c>
       <c r="B52" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B53" s="21" t="s">
-        <v>184</v>
-      </c>
-      <c r="C53" s="21"/>
+      <c r="B53" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="C53" s="22"/>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="B54" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="C54" s="22"/>
+        <v>134</v>
+      </c>
+      <c r="B54" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="C54" s="23"/>
     </row>
     <row r="55" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B55" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="C55" s="19"/>
+        <v>110</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="C55" s="20"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B56" s="8" t="s">
         <v>79</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="90" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B57" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B58" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C58" s="9" t="s">
         <v>162</v>
-      </c>
-      <c r="C58" s="9" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B59" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -2242,54 +2243,54 @@
     </row>
     <row r="2" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2325,13 +2326,13 @@
     </row>
     <row r="2" spans="1:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>80</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D2" s="14" t="str">
         <f>HYPERLINK(IF(RIGHT(CKAN_URL,1)="/", CKAN_URL &amp; "dataset/" &amp; package_name, CKAN_URL &amp; "/dataset/" &amp; package_name))</f>
@@ -2343,7 +2344,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>270</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>65</v>
@@ -2357,7 +2358,7 @@
         <v>58</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -2392,7 +2393,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -2400,7 +2401,7 @@
         <v>23</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -2408,7 +2409,7 @@
         <v>32</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -2416,7 +2417,7 @@
         <v>51</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -2424,7 +2425,7 @@
         <v>26</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2437,7 +2438,7 @@
         <v>28</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2447,13 +2448,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -2508,7 +2509,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -2529,19 +2530,19 @@
         <v>48</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="K1" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>208</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2558,7 +2559,7 @@
         <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -2567,10 +2568,10 @@
         <v>15</v>
       </c>
       <c r="I2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J2" t="s">
         <v>99</v>
-      </c>
-      <c r="J2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2587,36 +2588,36 @@
         <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
       </c>
       <c r="G3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="23" t="s">
-        <v>270</v>
+      <c r="L3" s="15" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D4" t="s">
         <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -2630,7 +2631,7 @@
         <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F5" t="s">
         <v>77</v>
@@ -2638,50 +2639,50 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D6" t="s">
+        <v>136</v>
+      </c>
+      <c r="F6" t="s">
         <v>115</v>
-      </c>
-      <c r="D6" t="s">
-        <v>137</v>
-      </c>
-      <c r="F6" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D7" t="s">
         <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
@@ -2689,42 +2690,45 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>124</v>
-      </c>
-      <c r="E9" t="s">
+        <v>123</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="F9" t="s">
         <v>168</v>
-      </c>
-      <c r="F9" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
       </c>
       <c r="D10" t="s">
+        <v>196</v>
+      </c>
+      <c r="E10" t="s">
+        <v>226</v>
+      </c>
+      <c r="F10" t="s">
         <v>197</v>
       </c>
-      <c r="E10" t="s">
-        <v>227</v>
-      </c>
-      <c r="F10" t="s">
-        <v>198</v>
-      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E9" r:id="rId1" xr:uid="{AE1B7623-EBDE-46E6-AAAF-66C8D56EA884}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2773,7 +2777,7 @@
         <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
@@ -2838,7 +2842,7 @@
         <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
@@ -2857,7 +2861,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>37</v>
@@ -2980,7 +2984,7 @@
         <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
@@ -3045,7 +3049,7 @@
         <v>21</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
@@ -3064,7 +3068,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>37</v>
@@ -3185,10 +3189,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="16"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -3201,10 +3205,10 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="15"/>
+      <c r="B6" s="16"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -3222,10 +3226,10 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="15"/>
+      <c r="B13" s="16"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -3244,54 +3248,54 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B19" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
+      <c r="A31" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="15"/>
+      <c r="B31" s="16"/>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -3311,14 +3315,14 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="B39" s="15"/>
+      <c r="B39" s="16"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
@@ -3333,7 +3337,7 @@
         <v>32</v>
       </c>
       <c r="B41" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -3349,128 +3353,128 @@
         <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>123</v>
+      </c>
+      <c r="B44" t="s">
         <v>124</v>
-      </c>
-      <c r="B44" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B45" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B46" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B47" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B48" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B49" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>224</v>
+      </c>
+      <c r="B50" t="s">
         <v>225</v>
-      </c>
-      <c r="B50" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>256</v>
+      </c>
+      <c r="B51" t="s">
         <v>257</v>
       </c>
-      <c r="B51" t="s">
-        <v>258</v>
-      </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="15" t="s">
-        <v>242</v>
-      </c>
-      <c r="B54" s="15"/>
+      <c r="A54" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="B54" s="16"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B56" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B57" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>246</v>
+      </c>
+      <c r="B58" t="s">
         <v>247</v>
-      </c>
-      <c r="B58" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>254</v>
+      </c>
+      <c r="B59" t="s">
         <v>255</v>
       </c>
-      <c r="B59" t="s">
-        <v>256</v>
-      </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="15" t="s">
+      <c r="A61" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B61" s="15"/>
+      <c r="B61" s="16"/>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>6</v>
       </c>
       <c r="B62" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -3478,35 +3482,35 @@
         <v>59</v>
       </c>
       <c r="B63" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>265</v>
+      </c>
+      <c r="B64" t="s">
         <v>266</v>
-      </c>
-      <c r="B64" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -3530,10 +3534,10 @@
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" s="15" t="s">
-        <v>253</v>
-      </c>
-      <c r="B78" s="15"/>
+      <c r="A78" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="B78" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
added: support for field units metadata in Excel file and CkanField objects fixed: view datastore_openlayers is optional
</commit_message>
<xml_diff>
--- a/src/ckanapi_harvesters/builder/builder_package_example.xlsx
+++ b/src/ckanapi_harvesters/builder/builder_package_example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\granierp\Projets\GPS_Mobilite_numerique\VRS_MobSciDatFactory\Repositories\ckanapi_harvesters\src\ckanapi_harvesters\builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{464EE3CE-8388-464C-B9A2-DE1DD6F8A970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11EC5A84-8020-4B93-B723-9C0C5F0FDAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{0974C446-06D1-4D56-994E-F584EC60B88C}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="275">
   <si>
     <t>Age of the individual</t>
   </si>
@@ -953,6 +953,18 @@
   </si>
   <si>
     <t>Example package to build with package builder from Python ckanapi_harvesters.builder</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>km/h</t>
+  </si>
+  <si>
+    <t>°</t>
+  </si>
+  <si>
+    <t>ISO-8601</t>
   </si>
 </sst>
 </file>
@@ -1077,6 +1089,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1101,7 +1114,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1560,25 +1572,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
     </row>
     <row r="2" spans="1:3" ht="102" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
     </row>
     <row r="3" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
@@ -1603,10 +1615,10 @@
       <c r="A7" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="20"/>
+      <c r="C7" s="21"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
@@ -1667,10 +1679,10 @@
       <c r="A13" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="C13" s="21"/>
+      <c r="C13" s="22"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
@@ -1841,10 +1853,10 @@
       <c r="A29" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="C29" s="20"/>
+      <c r="C29" s="21"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
@@ -1960,10 +1972,10 @@
       <c r="A40" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="C40" s="21"/>
+      <c r="C40" s="22"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
@@ -2101,28 +2113,28 @@
       <c r="A53" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B53" s="22" t="s">
+      <c r="B53" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="C53" s="22"/>
+      <c r="C53" s="23"/>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="B54" s="23" t="s">
+      <c r="B54" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="C54" s="23"/>
+      <c r="C54" s="24"/>
     </row>
     <row r="55" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B55" s="20" t="s">
+      <c r="B55" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="C55" s="20"/>
+      <c r="C55" s="21"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
@@ -2698,7 +2710,7 @@
       <c r="D9" t="s">
         <v>123</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="16" t="s">
         <v>167</v>
       </c>
       <c r="F9" t="s">
@@ -2824,7 +2836,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F87F6D0-62C0-4A6F-AD11-9303649DA230}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.85546875" style="1" customWidth="1"/>
@@ -2834,7 +2846,7 @@
     <col min="5" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>79</v>
       </c>
@@ -2847,8 +2859,11 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>73</v>
       </c>
@@ -2859,7 +2874,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>89</v>
       </c>
@@ -2870,7 +2885,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2881,7 +2896,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2891,8 +2906,11 @@
       <c r="D5" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="1" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>78</v>
       </c>
@@ -2902,8 +2920,11 @@
       <c r="D6" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="1" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
@@ -2913,8 +2934,11 @@
       <c r="D7" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
@@ -2924,8 +2948,11 @@
       <c r="D8" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>60</v>
       </c>
@@ -2935,8 +2962,11 @@
       <c r="D9" s="1" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" s="1" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -3189,10 +3219,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="16"/>
+      <c r="B2" s="17"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -3205,10 +3235,10 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="16"/>
+      <c r="B6" s="17"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -3226,10 +3256,10 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="17"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -3283,10 +3313,10 @@
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="16"/>
+      <c r="B31" s="17"/>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -3319,10 +3349,10 @@
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="16" t="s">
+      <c r="A39" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="B39" s="16"/>
+      <c r="B39" s="17"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
@@ -3421,10 +3451,10 @@
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="16" t="s">
+      <c r="A54" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="B54" s="16"/>
+      <c r="B54" s="17"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
@@ -3464,10 +3494,10 @@
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="16" t="s">
+      <c r="A61" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B61" s="16"/>
+      <c r="B61" s="17"/>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
@@ -3534,10 +3564,10 @@
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" s="16" t="s">
+      <c r="A78" s="17" t="s">
         <v>252</v>
       </c>
-      <c r="B78" s="16"/>
+      <c r="B78" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>